<commit_message>
Android: the page sits below the status bar
The status-bar plugin draws the page under the status bar by default,
but on Android 14 and older with a WebView before 140 nothing reports
the inset, so the header went under the clock (the smoke test's
screenshot). The page now sits below it, the bar in the page's color;
Android 15 and later already keep it clear. A device check is added.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ShQkzQ4P55GtAki1K96Y5n
</commit_message>
<xml_diff>
--- a/docs/device-test-results.xlsx
+++ b/docs/device-test-results.xlsx
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I58"/>
+  <dimension ref="A1:I59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1677,7 +1677,7 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>Android back button: closes an open menu (a song's, the sleep timer) or sheet first, then steps back through screens, and at the start puts the app in the background with the station still playing.</t>
+          <t>Android 14 or older: the header (the logo, Donate) sits below the status bar, never under the clock, in light and dark.</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
@@ -1712,19 +1712,54 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>First launch (delete and reinstall): the welcome appears once.</t>
-        </is>
-      </c>
-      <c r="C58" s="2" t="inlineStr"/>
-      <c r="D58" s="2" t="inlineStr"/>
-      <c r="E58" s="2" t="inlineStr"/>
-      <c r="F58" s="2" t="inlineStr"/>
+          <t>Android back button: closes an open menu (a song's, the sleep timer) or sheet first, then steps back through screens, and at the start puts the app in the background with the station still playing.</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="G58" s="2" t="inlineStr"/>
       <c r="H58" s="2" t="inlineStr"/>
       <c r="I58" s="2" t="inlineStr"/>
     </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>The system</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>First launch (delete and reinstall): the welcome appears once.</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr"/>
+      <c r="D59" s="2" t="inlineStr"/>
+      <c r="E59" s="2" t="inlineStr"/>
+      <c r="F59" s="2" t="inlineStr"/>
+      <c r="G59" s="2" t="inlineStr"/>
+      <c r="H59" s="2" t="inlineStr"/>
+      <c r="I59" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="C7:H58">
+  <conditionalFormatting sqref="C7:H59">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -1739,7 +1774,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="C7:H58" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C7:H59" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail,Blocked,N/A"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1798,23 +1833,23 @@
         </is>
       </c>
       <c r="B2">
-        <f>COUNTIF(Results!C7:C58,"Pass")</f>
+        <f>COUNTIF(Results!C7:C59,"Pass")</f>
         <v/>
       </c>
       <c r="C2">
-        <f>COUNTIF(Results!C7:C58,"Fail")</f>
+        <f>COUNTIF(Results!C7:C59,"Fail")</f>
         <v/>
       </c>
       <c r="D2">
-        <f>COUNTIF(Results!C7:C58,"Blocked")</f>
+        <f>COUNTIF(Results!C7:C59,"Blocked")</f>
         <v/>
       </c>
       <c r="E2">
-        <f>COUNTIF(Results!C7:C58,"N/A")</f>
+        <f>COUNTIF(Results!C7:C59,"N/A")</f>
         <v/>
       </c>
       <c r="F2">
-        <f>COUNTBLANK(Results!C7:C58)</f>
+        <f>COUNTBLANK(Results!C7:C59)</f>
         <v/>
       </c>
     </row>
@@ -1825,23 +1860,23 @@
         </is>
       </c>
       <c r="B3">
-        <f>COUNTIF(Results!D7:D58,"Pass")</f>
+        <f>COUNTIF(Results!D7:D59,"Pass")</f>
         <v/>
       </c>
       <c r="C3">
-        <f>COUNTIF(Results!D7:D58,"Fail")</f>
+        <f>COUNTIF(Results!D7:D59,"Fail")</f>
         <v/>
       </c>
       <c r="D3">
-        <f>COUNTIF(Results!D7:D58,"Blocked")</f>
+        <f>COUNTIF(Results!D7:D59,"Blocked")</f>
         <v/>
       </c>
       <c r="E3">
-        <f>COUNTIF(Results!D7:D58,"N/A")</f>
+        <f>COUNTIF(Results!D7:D59,"N/A")</f>
         <v/>
       </c>
       <c r="F3">
-        <f>COUNTBLANK(Results!D7:D58)</f>
+        <f>COUNTBLANK(Results!D7:D59)</f>
         <v/>
       </c>
     </row>
@@ -1852,23 +1887,23 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTIF(Results!E7:E58,"Pass")</f>
+        <f>COUNTIF(Results!E7:E59,"Pass")</f>
         <v/>
       </c>
       <c r="C4">
-        <f>COUNTIF(Results!E7:E58,"Fail")</f>
+        <f>COUNTIF(Results!E7:E59,"Fail")</f>
         <v/>
       </c>
       <c r="D4">
-        <f>COUNTIF(Results!E7:E58,"Blocked")</f>
+        <f>COUNTIF(Results!E7:E59,"Blocked")</f>
         <v/>
       </c>
       <c r="E4">
-        <f>COUNTIF(Results!E7:E58,"N/A")</f>
+        <f>COUNTIF(Results!E7:E59,"N/A")</f>
         <v/>
       </c>
       <c r="F4">
-        <f>COUNTBLANK(Results!E7:E58)</f>
+        <f>COUNTBLANK(Results!E7:E59)</f>
         <v/>
       </c>
     </row>
@@ -1879,23 +1914,23 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTIF(Results!F7:F58,"Pass")</f>
+        <f>COUNTIF(Results!F7:F59,"Pass")</f>
         <v/>
       </c>
       <c r="C5">
-        <f>COUNTIF(Results!F7:F58,"Fail")</f>
+        <f>COUNTIF(Results!F7:F59,"Fail")</f>
         <v/>
       </c>
       <c r="D5">
-        <f>COUNTIF(Results!F7:F58,"Blocked")</f>
+        <f>COUNTIF(Results!F7:F59,"Blocked")</f>
         <v/>
       </c>
       <c r="E5">
-        <f>COUNTIF(Results!F7:F58,"N/A")</f>
+        <f>COUNTIF(Results!F7:F59,"N/A")</f>
         <v/>
       </c>
       <c r="F5">
-        <f>COUNTBLANK(Results!F7:F58)</f>
+        <f>COUNTBLANK(Results!F7:F59)</f>
         <v/>
       </c>
     </row>
@@ -1906,23 +1941,23 @@
         </is>
       </c>
       <c r="B6">
-        <f>COUNTIF(Results!G7:G58,"Pass")</f>
+        <f>COUNTIF(Results!G7:G59,"Pass")</f>
         <v/>
       </c>
       <c r="C6">
-        <f>COUNTIF(Results!G7:G58,"Fail")</f>
+        <f>COUNTIF(Results!G7:G59,"Fail")</f>
         <v/>
       </c>
       <c r="D6">
-        <f>COUNTIF(Results!G7:G58,"Blocked")</f>
+        <f>COUNTIF(Results!G7:G59,"Blocked")</f>
         <v/>
       </c>
       <c r="E6">
-        <f>COUNTIF(Results!G7:G58,"N/A")</f>
+        <f>COUNTIF(Results!G7:G59,"N/A")</f>
         <v/>
       </c>
       <c r="F6">
-        <f>COUNTBLANK(Results!G7:G58)</f>
+        <f>COUNTBLANK(Results!G7:G59)</f>
         <v/>
       </c>
     </row>
@@ -1933,23 +1968,23 @@
         </is>
       </c>
       <c r="B7">
-        <f>COUNTIF(Results!H7:H58,"Pass")</f>
+        <f>COUNTIF(Results!H7:H59,"Pass")</f>
         <v/>
       </c>
       <c r="C7">
-        <f>COUNTIF(Results!H7:H58,"Fail")</f>
+        <f>COUNTIF(Results!H7:H59,"Fail")</f>
         <v/>
       </c>
       <c r="D7">
-        <f>COUNTIF(Results!H7:H58,"Blocked")</f>
+        <f>COUNTIF(Results!H7:H59,"Blocked")</f>
         <v/>
       </c>
       <c r="E7">
-        <f>COUNTIF(Results!H7:H58,"N/A")</f>
+        <f>COUNTIF(Results!H7:H59,"N/A")</f>
         <v/>
       </c>
       <c r="F7">
-        <f>COUNTBLANK(Results!H7:H58)</f>
+        <f>COUNTBLANK(Results!H7:H59)</f>
         <v/>
       </c>
     </row>

</xml_diff>